<commit_message>
added new data for OPM 2026
</commit_message>
<xml_diff>
--- a/data/Oficina_de_procuradora_de_mujeres/opmAgresores.xlsx
+++ b/data/Oficina_de_procuradora_de_mujeres/opmAgresores.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gnper\Documents\ViolenciaGeneroPR\data\Oficina_de_procuradora_de_mujeres\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B731E979-6EEE-456F-923F-442E2D677181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E3566C5-A868-4395-9226-A79AC4DF4397}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5880" yWindow="2196" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="10">
   <si>
     <t>year</t>
   </si>
@@ -383,7 +383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24.109375" bestFit="1" customWidth="1"/>
@@ -631,6 +631,83 @@
         <v>0</v>
       </c>
     </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>2026</v>
+      </c>
+      <c r="B23" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>2026</v>
+      </c>
+      <c r="B24" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>2026</v>
+      </c>
+      <c r="B25" t="s">
+        <v>5</v>
+      </c>
+      <c r="C25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>2026</v>
+      </c>
+      <c r="B26" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>2026</v>
+      </c>
+      <c r="B27" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>2026</v>
+      </c>
+      <c r="B28" t="s">
+        <v>8</v>
+      </c>
+      <c r="C28">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>2026</v>
+      </c>
+      <c r="B29" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>